<commit_message>
completed curated transformation and testing
</commit_message>
<xml_diff>
--- a/documentation/testing/Unit Test Cases.xlsx
+++ b/documentation/testing/Unit Test Cases.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\devInsureDataPipeline\documentation\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{232C5280-84E1-4E83-99AD-C79B6A14A47F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3867574E-F1EC-4C60-834E-FF9197C9942A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="62">
   <si>
     <t>Object_name</t>
   </si>
   <si>
-    <t>Test case Numbr</t>
-  </si>
-  <si>
     <t>Scenario</t>
   </si>
   <si>
@@ -139,6 +136,60 @@
   </si>
   <si>
     <t>Verify that a validated CSV file is successfully converted into a Parquet file and stored in the preprocessed folder</t>
+  </si>
+  <si>
+    <t>Validated CSV file was successfully converted to Parquet and stored in the preprocessed folder.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass </t>
+  </si>
+  <si>
+    <t>Duplicate row removal</t>
+  </si>
+  <si>
+    <t>Verify that duplicate rows are removed from the validated CSV during preprocessing.</t>
+  </si>
+  <si>
+    <t>Duplicate rows should removed and only unique rows should remain</t>
+  </si>
+  <si>
+    <t>Duplicate Rows removed Successfully, only unique rows remains</t>
+  </si>
+  <si>
+    <t>Ingestion date addition</t>
+  </si>
+  <si>
+    <t>Verify that the current system date and time is added to the ingestion_date column during preprocessing.</t>
+  </si>
+  <si>
+    <t>The processed data should contain an ingestion_date column with the current processing date and time.</t>
+  </si>
+  <si>
+    <t>ingestion_date column was successfully added with the current processing timestamp.</t>
+  </si>
+  <si>
+    <t>File date extraction</t>
+  </si>
+  <si>
+    <t>Verify that the date from the validated filename is correctly extracted and added to the file_date column.</t>
+  </si>
+  <si>
+    <t>The YYYYMMDD date from the filename should be converted to a valid date and added to file_date.</t>
+  </si>
+  <si>
+    <t>File date 20260815 was successfully converted to 2026-08-15 and added to file_date.</t>
+  </si>
+  <si>
+    <t>Multiple Validated Files Processing</t>
+  </si>
+  <si>
+    <t>varify that all files available in the validated_files folder are processed individually and converted to parquet</t>
+  </si>
+  <si>
+    <t>All validated CSV files should be processed successfully and corresponding parquet files should be created in the preprocessed folder</t>
+  </si>
+  <si>
+    <t>All validated files were processed successfully and correspondiong parquet files were created</t>
   </si>
   <si>
     <r>
@@ -146,7 +197,7 @@
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
+        <sz val="14"/>
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
@@ -154,74 +205,30 @@
     </r>
   </si>
   <si>
-    <t>Validated CSV file was successfully converted to Parquet and stored in the preprocessed folder.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pass </t>
-  </si>
-  <si>
-    <t>Duplicate row removal</t>
-  </si>
-  <si>
-    <t>Verify that duplicate rows are removed from the validated CSV during preprocessing.</t>
-  </si>
-  <si>
-    <t>Duplicate rows should removed and only unique rows should remain</t>
-  </si>
-  <si>
-    <t>Duplicate Rows removed Successfully, only unique rows remains</t>
-  </si>
-  <si>
-    <t>Ingestion date addition</t>
-  </si>
-  <si>
-    <t>Verify that the current system date and time is added to the ingestion_date column during preprocessing.</t>
-  </si>
-  <si>
-    <t>The processed data should contain an ingestion_date column with the current processing date and time.</t>
-  </si>
-  <si>
-    <t>ingestion_date column was successfully added with the current processing timestamp.</t>
-  </si>
-  <si>
-    <t>File date extraction</t>
-  </si>
-  <si>
-    <t>Verify that the date from the validated filename is correctly extracted and added to the file_date column.</t>
-  </si>
-  <si>
-    <t>The YYYYMMDD date from the filename should be converted to a valid date and added to file_date.</t>
-  </si>
-  <si>
-    <t>File date 20260815 was successfully converted to 2026-08-15 and added to file_date.</t>
-  </si>
-  <si>
-    <t>Multiple Validated Files Processing</t>
-  </si>
-  <si>
-    <t>varify that all files available in the validated_files folder are processed individually and converted to parquet</t>
-  </si>
-  <si>
-    <t>All validated CSV files should be processed successfully and corresponding parquet files should be created in the preprocessed folder</t>
-  </si>
-  <si>
-    <t>All validated files were processed successfully and correspondiong parquet files were created</t>
+    <t>Test case Number</t>
+  </si>
+  <si>
+    <t>transformation_engine</t>
+  </si>
+  <si>
+    <t>Curated Output Creation</t>
+  </si>
+  <si>
+    <t>Varify that the curated transformation creates the required curated parquet file with the required columns</t>
+  </si>
+  <si>
+    <t>Curated parquet file should be created successfully and should contain the required curated columns</t>
+  </si>
+  <si>
+    <t>Curated parquet files was created successfully and contained the required curated columns</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -240,13 +247,28 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
@@ -265,7 +287,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -288,66 +310,61 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -379,7 +396,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>11906</xdr:colOff>
+      <xdr:colOff>11907</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>2750343</xdr:rowOff>
     </xdr:to>
@@ -428,7 +445,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>1</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>2690812</xdr:rowOff>
     </xdr:to>
@@ -528,7 +545,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>23813</xdr:colOff>
+      <xdr:colOff>23814</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2821781</xdr:rowOff>
     </xdr:to>
@@ -578,7 +595,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>59531</xdr:colOff>
+      <xdr:colOff>59532</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>11905</xdr:rowOff>
     </xdr:to>
@@ -628,7 +645,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>11906</xdr:colOff>
+      <xdr:colOff>11907</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -678,7 +695,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:colOff>2</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2702719</xdr:rowOff>
     </xdr:to>
@@ -728,7 +745,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>59532</xdr:colOff>
+      <xdr:colOff>59533</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>29767</xdr:rowOff>
     </xdr:to>
@@ -778,7 +795,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>12370</xdr:colOff>
+      <xdr:colOff>12371</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -828,7 +845,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>21167</xdr:colOff>
+      <xdr:colOff>21168</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>21167</xdr:rowOff>
     </xdr:to>
@@ -878,7 +895,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>1</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -911,6 +928,56 @@
         <a:xfrm>
           <a:off x="11246827" y="27878942"/>
           <a:ext cx="3993173" cy="3443654"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>77230</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0C59C3C9-B465-BA4E-5F25-F3DC4A1F4BE2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13257770" y="31226555"/>
+          <a:ext cx="4067433" cy="3089188"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1185,487 +1252,463 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:Z16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.5703125" customWidth="1"/>
     <col min="2" max="2" width="22.28515625" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="30.42578125" customWidth="1"/>
+    <col min="5" max="5" width="28.42578125" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" customWidth="1"/>
     <col min="7" max="7" width="15.28515625" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" customWidth="1"/>
     <col min="9" max="9" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:26" ht="18.75">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+    </row>
+    <row r="2" spans="1:26" ht="182.25" customHeight="1">
+      <c r="A2" s="14" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="15"/>
-      <c r="T1" s="15"/>
-      <c r="U1" s="15"/>
-      <c r="V1" s="15"/>
-      <c r="W1" s="15"/>
-      <c r="X1" s="15"/>
-      <c r="Y1" s="15"/>
-      <c r="Z1" s="15"/>
-      <c r="AA1" s="16"/>
-      <c r="AB1" s="16"/>
-      <c r="AC1" s="16"/>
-    </row>
-    <row r="2" spans="1:29" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>9</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="9" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="H2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="10"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="17"/>
-      <c r="S2" s="17"/>
-      <c r="T2" s="17"/>
-      <c r="U2" s="17"/>
-      <c r="V2" s="17"/>
-      <c r="W2" s="17"/>
-      <c r="X2" s="17"/>
-      <c r="Y2" s="17"/>
-      <c r="Z2" s="17"/>
-      <c r="AA2" s="16"/>
-      <c r="AB2" s="16"/>
-      <c r="AC2" s="16"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
     </row>
-    <row r="3" spans="1:29" ht="218.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
+    <row r="3" spans="1:26" ht="218.25" customHeight="1">
+      <c r="A3" s="14"/>
       <c r="B3" s="4">
         <v>2</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="E3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="10"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-      <c r="W3" s="17"/>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="17"/>
-      <c r="AA3" s="16"/>
-      <c r="AB3" s="16"/>
-      <c r="AC3" s="16"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:29" ht="213.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
+    <row r="4" spans="1:26" ht="213.75" customHeight="1">
+      <c r="A4" s="14"/>
       <c r="B4" s="4">
         <v>3</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="G4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="10"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
-      <c r="R4" s="17"/>
-      <c r="S4" s="17"/>
-      <c r="T4" s="17"/>
-      <c r="U4" s="17"/>
-      <c r="V4" s="17"/>
-      <c r="W4" s="17"/>
-      <c r="X4" s="17"/>
-      <c r="Y4" s="17"/>
-      <c r="Z4" s="17"/>
-      <c r="AA4" s="16"/>
-      <c r="AB4" s="16"/>
-      <c r="AC4" s="16"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
     </row>
-    <row r="5" spans="1:29" ht="224.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6"/>
+    <row r="5" spans="1:26" ht="224.25" customHeight="1">
+      <c r="A5" s="14"/>
       <c r="B5" s="4">
         <v>4</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="E5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>26</v>
-      </c>
       <c r="G5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="13"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="17"/>
-      <c r="R5" s="17"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="17"/>
-      <c r="U5" s="17"/>
-      <c r="V5" s="17"/>
-      <c r="W5" s="17"/>
-      <c r="X5" s="17"/>
-      <c r="Y5" s="17"/>
-      <c r="Z5" s="17"/>
-      <c r="AA5" s="16"/>
-      <c r="AB5" s="16"/>
-      <c r="AC5" s="16"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
     </row>
-    <row r="6" spans="1:29" ht="237" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
+    <row r="6" spans="1:26" ht="237" customHeight="1">
+      <c r="A6" s="14"/>
       <c r="B6" s="4">
         <v>5</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="E6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="6"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="1"/>
+      <c r="Z6" s="1"/>
+    </row>
+    <row r="7" spans="1:26" ht="252" customHeight="1">
+      <c r="A7" s="14"/>
+      <c r="B7" s="9">
+        <v>6</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="D7" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="10"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
-      <c r="S6" s="15"/>
-      <c r="T6" s="15"/>
-      <c r="U6" s="15"/>
-      <c r="V6" s="15"/>
-      <c r="W6" s="15"/>
-      <c r="X6" s="15"/>
-      <c r="Y6" s="15"/>
-      <c r="Z6" s="15"/>
-      <c r="AA6" s="16"/>
-      <c r="AB6" s="16"/>
-      <c r="AC6" s="16"/>
+      <c r="I7" s="4"/>
     </row>
-    <row r="7" spans="1:29" ht="252" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="1">
-        <v>6</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="3" t="s">
+    <row r="8" spans="1:26" ht="213.75" customHeight="1">
+      <c r="A8" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="B8" s="4">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="8"/>
+    </row>
+    <row r="9" spans="1:26" ht="187.5" customHeight="1">
+      <c r="A9" s="15"/>
+      <c r="B9" s="4">
+        <v>8</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="16"/>
-      <c r="U7" s="16"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="16"/>
-      <c r="X7" s="16"/>
-      <c r="Y7" s="16"/>
-      <c r="Z7" s="16"/>
-      <c r="AA7" s="16"/>
-      <c r="AB7" s="16"/>
-      <c r="AC7" s="16"/>
+      <c r="I9" s="8"/>
     </row>
-    <row r="8" spans="1:29" ht="213.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="18">
-        <v>7</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" s="18" t="s">
+    <row r="10" spans="1:26" ht="214.5" customHeight="1">
+      <c r="A10" s="15"/>
+      <c r="B10" s="4">
+        <v>9</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="13"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="16"/>
-      <c r="U8" s="16"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="16"/>
-      <c r="X8" s="16"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="16"/>
-      <c r="AA8" s="16"/>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="16"/>
+      <c r="I10" s="8"/>
     </row>
-    <row r="9" spans="1:29" ht="187.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="18">
-        <v>8</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="18" t="s">
+    <row r="11" spans="1:26" ht="225.75" customHeight="1">
+      <c r="A11" s="15"/>
+      <c r="B11" s="4">
+        <v>10</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="13"/>
+      <c r="I11" s="8"/>
     </row>
-    <row r="10" spans="1:29" ht="214.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" s="18">
-        <v>9</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G10" s="18" t="s">
+    <row r="12" spans="1:26" ht="270.75" customHeight="1">
+      <c r="A12" s="15"/>
+      <c r="B12" s="4">
+        <v>11</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" s="13"/>
+      <c r="I12" s="8"/>
     </row>
-    <row r="11" spans="1:29" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
-      <c r="B11" s="18">
-        <v>10</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G11" s="18" t="s">
+    <row r="13" spans="1:26" ht="243.75" customHeight="1">
+      <c r="A13" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="9">
+        <v>12</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" s="13"/>
+      <c r="I13" s="8"/>
     </row>
-    <row r="12" spans="1:29" ht="270.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="21"/>
-      <c r="B12" s="18">
-        <v>11</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="F12" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="G12" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" s="13"/>
+    <row r="14" spans="1:26" ht="18.75">
+      <c r="B14" s="13"/>
+    </row>
+    <row r="16" spans="1:26">
+      <c r="H16" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
sementic layer coding and testing completed
</commit_message>
<xml_diff>
--- a/documentation/testing/Unit Test Cases.xlsx
+++ b/documentation/testing/Unit Test Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\devInsureDataPipeline\documentation\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3867574E-F1EC-4C60-834E-FF9197C9942A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2347B8A9-9681-4F9F-8FCC-90ACF89D9C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="66">
   <si>
     <t>Object_name</t>
   </si>
@@ -221,6 +221,92 @@
   </si>
   <si>
     <t>Curated parquet files was created successfully and contained the required curated columns</t>
+  </si>
+  <si>
+    <t>Verify Semantic Layer output</t>
+  </si>
+  <si>
+    <t>Verify that the Curated data is successfully aggregated by Policy_Type and the Semantic output file is created with the required columns</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Semantic file should be created successfully at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>data/semantic/PolicyTypeAgg.parquet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Policy_Type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>avg_claim_amount</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>count_claims</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> columns and should contain aggregated data</t>
+    </r>
+  </si>
+  <si>
+    <t>Semantic file was successfully created with 5 rows and the required columns Policy_Type, avg_claim_amount, and count_claims</t>
   </si>
 </sst>
 </file>
@@ -287,7 +373,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -321,12 +407,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -352,9 +458,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -365,6 +468,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -978,6 +1096,56 @@
         <a:xfrm>
           <a:off x="13257770" y="31226555"/>
           <a:ext cx="4067433" cy="3089188"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>32845</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5205745-382E-469D-48C0-913A086A92DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13187198" y="34322846"/>
+          <a:ext cx="4039914" cy="3826422"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1314,13 +1482,13 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="182.25" customHeight="1">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="13" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="7" t="s">
@@ -1358,7 +1526,7 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" spans="1:26" ht="218.25" customHeight="1">
-      <c r="A3" s="14"/>
+      <c r="A3" s="13"/>
       <c r="B3" s="4">
         <v>2</v>
       </c>
@@ -1400,7 +1568,7 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" spans="1:26" ht="213.75" customHeight="1">
-      <c r="A4" s="14"/>
+      <c r="A4" s="13"/>
       <c r="B4" s="4">
         <v>3</v>
       </c>
@@ -1442,7 +1610,7 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5" spans="1:26" ht="224.25" customHeight="1">
-      <c r="A5" s="14"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="4">
         <v>4</v>
       </c>
@@ -1484,7 +1652,7 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6" spans="1:26" ht="237" customHeight="1">
-      <c r="A6" s="14"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="4">
         <v>5</v>
       </c>
@@ -1526,7 +1694,7 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="252" customHeight="1">
-      <c r="A7" s="14"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="9">
         <v>6</v>
       </c>
@@ -1551,7 +1719,7 @@
       <c r="I7" s="4"/>
     </row>
     <row r="8" spans="1:26" ht="213.75" customHeight="1">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="14" t="s">
         <v>34</v>
       </c>
       <c r="B8" s="4">
@@ -1578,7 +1746,7 @@
       <c r="I8" s="8"/>
     </row>
     <row r="9" spans="1:26" ht="187.5" customHeight="1">
-      <c r="A9" s="15"/>
+      <c r="A9" s="14"/>
       <c r="B9" s="4">
         <v>8</v>
       </c>
@@ -1603,7 +1771,7 @@
       <c r="I9" s="8"/>
     </row>
     <row r="10" spans="1:26" ht="214.5" customHeight="1">
-      <c r="A10" s="15"/>
+      <c r="A10" s="14"/>
       <c r="B10" s="4">
         <v>9</v>
       </c>
@@ -1628,7 +1796,7 @@
       <c r="I10" s="8"/>
     </row>
     <row r="11" spans="1:26" ht="225.75" customHeight="1">
-      <c r="A11" s="15"/>
+      <c r="A11" s="14"/>
       <c r="B11" s="4">
         <v>10</v>
       </c>
@@ -1653,7 +1821,7 @@
       <c r="I11" s="8"/>
     </row>
     <row r="12" spans="1:26" ht="270.75" customHeight="1">
-      <c r="A12" s="15"/>
+      <c r="A12" s="14"/>
       <c r="B12" s="4">
         <v>11</v>
       </c>
@@ -1678,7 +1846,7 @@
       <c r="I12" s="8"/>
     </row>
     <row r="13" spans="1:26" ht="243.75" customHeight="1">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="15" t="s">
         <v>57</v>
       </c>
       <c r="B13" s="9">
@@ -1704,16 +1872,38 @@
       </c>
       <c r="I13" s="8"/>
     </row>
-    <row r="14" spans="1:26" ht="18.75">
-      <c r="B14" s="13"/>
+    <row r="14" spans="1:26" ht="300.75" customHeight="1">
+      <c r="A14" s="16"/>
+      <c r="B14" s="12">
+        <v>13</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="19" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="16" spans="1:26">
       <c r="H16" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:A7"/>
     <mergeCell ref="A8:A12"/>
+    <mergeCell ref="A13:A14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>